<commit_message>
Canada capacity: StatCan 'Total thermal' includes nuclear steam - subtract it before the by-fuel remainder (nuclear was double counted in Other); saved workbook corrected
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HgApe3mo6LmJKGvZpZM695
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/canada_power_capacity.xlsx
+++ b/output/Data and Chart Outputs/canada_power_capacity.xlsx
@@ -944,7 +944,7 @@
         <v>8.3725</v>
       </c>
       <c r="I2" t="n">
-        <v>32.806</v>
+        <v>18.303</v>
       </c>
     </row>
     <row r="3">
@@ -973,7 +973,7 @@
         <v>4.4845</v>
       </c>
       <c r="I3" t="n">
-        <v>32.7265</v>
+        <v>18.2235</v>
       </c>
     </row>
     <row r="4">
@@ -1002,7 +1002,7 @@
         <v>4.0785</v>
       </c>
       <c r="I4" t="n">
-        <v>30.3495</v>
+        <v>17.0535</v>
       </c>
     </row>
     <row r="5">
@@ -1031,7 +1031,7 @@
         <v>3.2155</v>
       </c>
       <c r="I5" t="n">
-        <v>31.9452</v>
+        <v>17.7602</v>
       </c>
     </row>
   </sheetData>
@@ -1127,7 +1127,7 @@
         <v>5947.3</v>
       </c>
       <c r="I2" t="n">
-        <v>17846.9</v>
+        <v>3745.9</v>
       </c>
       <c r="J2" t="n">
         <v>145537.8</v>
@@ -1159,7 +1159,7 @@
         <v>5947.7</v>
       </c>
       <c r="I3" t="n">
-        <v>17918.4</v>
+        <v>3817.4</v>
       </c>
       <c r="J3" t="n">
         <v>145960.9</v>
@@ -1191,7 +1191,7 @@
         <v>5930.3</v>
       </c>
       <c r="I4" t="n">
-        <v>18303</v>
+        <v>3800</v>
       </c>
       <c r="J4" t="n">
         <v>149530.5</v>
@@ -1223,7 +1223,7 @@
         <v>5773.4</v>
       </c>
       <c r="I5" t="n">
-        <v>18223.5</v>
+        <v>3720.5</v>
       </c>
       <c r="J5" t="n">
         <v>151706.7</v>
@@ -1255,7 +1255,7 @@
         <v>5778.4</v>
       </c>
       <c r="I6" t="n">
-        <v>17053.5</v>
+        <v>3757.5</v>
       </c>
       <c r="J6" t="n">
         <v>150937.7</v>
@@ -1287,7 +1287,7 @@
         <v>5724.4</v>
       </c>
       <c r="I7" t="n">
-        <v>17760.2</v>
+        <v>3575.2</v>
       </c>
       <c r="J7" t="n">
         <v>156388.5</v>

</xml_diff>